<commit_message>
lot of changes, mainly adding log file for mutation and extractig info from xlsx file
</commit_message>
<xml_diff>
--- a/New_Code/mutation.xlsx
+++ b/New_Code/mutation.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Guillaume\Desktop\hERG\New_Code\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B73E785-715C-483D-BA76-747EB8358DBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6754C989-4E36-400E-89A6-753547E7B93F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{25DD2874-44EC-4C00-8F62-207BA1D39B57}"/>
+    <workbookView xWindow="15810" yWindow="1485" windowWidth="12000" windowHeight="11295" xr2:uid="{25DD2874-44EC-4C00-8F62-207BA1D39B57}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -36,13 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
-  <si>
-    <t>Y248T</t>
-  </si>
-  <si>
-    <t>A123G</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
     <t>critère1</t>
   </si>
@@ -59,7 +53,16 @@
     <t>AA_important en contact</t>
   </si>
   <si>
-    <t>P489R</t>
+    <t>clash</t>
+  </si>
+  <si>
+    <t>critère4</t>
+  </si>
+  <si>
+    <t>total</t>
+  </si>
+  <si>
+    <t>L839T</t>
   </si>
 </sst>
 </file>
@@ -411,46 +414,55 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5762739B-326A-4783-9A65-DF487FD1A3E8}">
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="7" width="30.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>0</v>
       </c>
-      <c r="C1" t="s">
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>1</v>
       </c>
-      <c r="D1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
         <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
ajout de la lecture et l'écriture dans le fichier mutation.xlsx
</commit_message>
<xml_diff>
--- a/New_Code/mutation.xlsx
+++ b/New_Code/mutation.xlsx
@@ -8,35 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Guillaume\Desktop\hERG\New_Code\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6754C989-4E36-400E-89A6-753547E7B93F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9EE7A5A8-C747-4DF7-9E76-96C09DC55EBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15810" yWindow="1485" windowWidth="12000" windowHeight="11295" xr2:uid="{25DD2874-44EC-4C00-8F62-207BA1D39B57}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>critère1</t>
   </si>
@@ -47,13 +31,10 @@
     <t>critère3</t>
   </si>
   <si>
-    <t>minimisation</t>
+    <t>clash</t>
   </si>
   <si>
-    <t>AA_important en contact</t>
-  </si>
-  <si>
-    <t>clash</t>
+    <t>minimisation</t>
   </si>
   <si>
     <t>critère4</t>
@@ -62,14 +43,14 @@
     <t>total</t>
   </si>
   <si>
-    <t>L839T</t>
+    <t>AA_important en contact</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -77,16 +58,322 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="Calibri Light"/>
+      <family val="2"/>
+      <scheme val="major"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="34">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.59999389629810485"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.39997558519241921"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.59999389629810485"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.39997558519241921"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.79998168889431442"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.59999389629810485"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.39997558519241921"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.79998168889431442"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.59999389629810485"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.39997558519241921"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.79998168889431442"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.59999389629810485"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.39997558519241921"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.39997558519241921"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -94,15 +381,233 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thick">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thick">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="12" borderId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="16" borderId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="20" borderId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="24" borderId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="28" borderId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="32" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="4"/>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="5"/>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="4"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="6"/>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="7"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="8"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="9"/>
+    <xf numFmtId="0" fontId="16" fillId="9" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="11" borderId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="12" borderId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="13" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="14" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="15" borderId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="16" borderId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="17" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="18" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="19" borderId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="20" borderId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="21" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="22" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="23" borderId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="24" borderId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="25" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="26" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="27" borderId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="28" borderId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="29" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="30" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="31" borderId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="32" borderId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="12" borderId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="16" borderId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="20" borderId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="24" borderId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="28" borderId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="32" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="56">
+    <cellStyle name="20 % - Accent1 2" xfId="26" xr:uid="{00000000-0005-0000-0000-00001A000000}"/>
+    <cellStyle name="20 % - Accent2 2" xfId="30" xr:uid="{00000000-0005-0000-0000-00001E000000}"/>
+    <cellStyle name="20 % - Accent3 2" xfId="34" xr:uid="{00000000-0005-0000-0000-000022000000}"/>
+    <cellStyle name="20 % - Accent4 2" xfId="38" xr:uid="{00000000-0005-0000-0000-000026000000}"/>
+    <cellStyle name="20 % - Accent5 2" xfId="42" xr:uid="{00000000-0005-0000-0000-00002A000000}"/>
+    <cellStyle name="20 % - Accent6 2" xfId="46" xr:uid="{00000000-0005-0000-0000-00002E000000}"/>
+    <cellStyle name="40 % - Accent1 2" xfId="27" xr:uid="{00000000-0005-0000-0000-00001B000000}"/>
+    <cellStyle name="40 % - Accent2 2" xfId="31" xr:uid="{00000000-0005-0000-0000-00001F000000}"/>
+    <cellStyle name="40 % - Accent3 2" xfId="35" xr:uid="{00000000-0005-0000-0000-000023000000}"/>
+    <cellStyle name="40 % - Accent4 2" xfId="39" xr:uid="{00000000-0005-0000-0000-000027000000}"/>
+    <cellStyle name="40 % - Accent5 2" xfId="43" xr:uid="{00000000-0005-0000-0000-00002B000000}"/>
+    <cellStyle name="40 % - Accent6 2" xfId="47" xr:uid="{00000000-0005-0000-0000-00002F000000}"/>
+    <cellStyle name="60 % - Accent1 2" xfId="2" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
+    <cellStyle name="60 % - Accent1 3" xfId="28" xr:uid="{00000000-0005-0000-0000-00001C000000}"/>
+    <cellStyle name="60 % - Accent1 4" xfId="50" xr:uid="{00000000-0005-0000-0000-000054000000}"/>
+    <cellStyle name="60 % - Accent2 2" xfId="3" xr:uid="{00000000-0005-0000-0000-000003000000}"/>
+    <cellStyle name="60 % - Accent2 3" xfId="32" xr:uid="{00000000-0005-0000-0000-000020000000}"/>
+    <cellStyle name="60 % - Accent2 4" xfId="51" xr:uid="{00000000-0005-0000-0000-000055000000}"/>
+    <cellStyle name="60 % - Accent3 2" xfId="4" xr:uid="{00000000-0005-0000-0000-000004000000}"/>
+    <cellStyle name="60 % - Accent3 3" xfId="36" xr:uid="{00000000-0005-0000-0000-000024000000}"/>
+    <cellStyle name="60 % - Accent3 4" xfId="52" xr:uid="{00000000-0005-0000-0000-000056000000}"/>
+    <cellStyle name="60 % - Accent4 2" xfId="5" xr:uid="{00000000-0005-0000-0000-000005000000}"/>
+    <cellStyle name="60 % - Accent4 3" xfId="40" xr:uid="{00000000-0005-0000-0000-000028000000}"/>
+    <cellStyle name="60 % - Accent4 4" xfId="53" xr:uid="{00000000-0005-0000-0000-000057000000}"/>
+    <cellStyle name="60 % - Accent5 2" xfId="6" xr:uid="{00000000-0005-0000-0000-000006000000}"/>
+    <cellStyle name="60 % - Accent5 3" xfId="44" xr:uid="{00000000-0005-0000-0000-00002C000000}"/>
+    <cellStyle name="60 % - Accent5 4" xfId="54" xr:uid="{00000000-0005-0000-0000-000058000000}"/>
+    <cellStyle name="60 % - Accent6 2" xfId="7" xr:uid="{00000000-0005-0000-0000-000007000000}"/>
+    <cellStyle name="60 % - Accent6 3" xfId="48" xr:uid="{00000000-0005-0000-0000-000030000000}"/>
+    <cellStyle name="60 % - Accent6 4" xfId="55" xr:uid="{00000000-0005-0000-0000-000059000000}"/>
+    <cellStyle name="Accent1 2" xfId="25" xr:uid="{00000000-0005-0000-0000-000019000000}"/>
+    <cellStyle name="Accent2 2" xfId="29" xr:uid="{00000000-0005-0000-0000-00001D000000}"/>
+    <cellStyle name="Accent3 2" xfId="33" xr:uid="{00000000-0005-0000-0000-000021000000}"/>
+    <cellStyle name="Accent4 2" xfId="37" xr:uid="{00000000-0005-0000-0000-000025000000}"/>
+    <cellStyle name="Accent5 2" xfId="41" xr:uid="{00000000-0005-0000-0000-000029000000}"/>
+    <cellStyle name="Accent6 2" xfId="45" xr:uid="{00000000-0005-0000-0000-00002D000000}"/>
+    <cellStyle name="Avertissement 2" xfId="21" xr:uid="{00000000-0005-0000-0000-000015000000}"/>
+    <cellStyle name="Calcul 2" xfId="18" xr:uid="{00000000-0005-0000-0000-000012000000}"/>
+    <cellStyle name="Cellule liée 2" xfId="19" xr:uid="{00000000-0005-0000-0000-000013000000}"/>
+    <cellStyle name="Entrée 2" xfId="16" xr:uid="{00000000-0005-0000-0000-000010000000}"/>
+    <cellStyle name="Insatisfaisant 2" xfId="14" xr:uid="{00000000-0005-0000-0000-00000E000000}"/>
+    <cellStyle name="Neutre 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
+    <cellStyle name="Neutre 3" xfId="15" xr:uid="{00000000-0005-0000-0000-00000F000000}"/>
+    <cellStyle name="Neutre 4" xfId="49" xr:uid="{00000000-0005-0000-0000-000053000000}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Note 2" xfId="22" xr:uid="{00000000-0005-0000-0000-000016000000}"/>
+    <cellStyle name="Satisfaisant 2" xfId="13" xr:uid="{00000000-0005-0000-0000-00000D000000}"/>
+    <cellStyle name="Sortie 2" xfId="17" xr:uid="{00000000-0005-0000-0000-000011000000}"/>
+    <cellStyle name="Texte explicatif 2" xfId="23" xr:uid="{00000000-0005-0000-0000-000017000000}"/>
+    <cellStyle name="Titre 2" xfId="8" xr:uid="{00000000-0005-0000-0000-000008000000}"/>
+    <cellStyle name="Titre 1 2" xfId="9" xr:uid="{00000000-0005-0000-0000-000009000000}"/>
+    <cellStyle name="Titre 2 2" xfId="10" xr:uid="{00000000-0005-0000-0000-00000A000000}"/>
+    <cellStyle name="Titre 3 2" xfId="11" xr:uid="{00000000-0005-0000-0000-00000B000000}"/>
+    <cellStyle name="Titre 4 2" xfId="12" xr:uid="{00000000-0005-0000-0000-00000C000000}"/>
+    <cellStyle name="Total 2" xfId="24" xr:uid="{00000000-0005-0000-0000-000018000000}"/>
+    <cellStyle name="Vérification 2" xfId="20" xr:uid="{00000000-0005-0000-0000-000014000000}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -413,56 +918,54 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5762739B-326A-4783-9A65-DF487FD1A3E8}">
-  <dimension ref="A1:B9"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="7" width="30.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B1" t="s">
-        <v>8</v>
-      </c>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="F1" s="1"/>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
         <v>7</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
functional version, needs stress test
</commit_message>
<xml_diff>
--- a/New_Code/mutation.xlsx
+++ b/New_Code/mutation.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Guillaume\Desktop\hERG\New_Code\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9EE7A5A8-C747-4DF7-9E76-96C09DC55EBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{522CAF5F-2570-4497-88C7-62C6CA3C1DCF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -489,7 +489,7 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="56">
+  <cellStyleXfs count="77">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="17" fillId="4" borderId="0"/>
     <xf numFmtId="0" fontId="16" fillId="12" borderId="0"/>
@@ -546,12 +546,33 @@
     <xf numFmtId="0" fontId="16" fillId="24" borderId="0"/>
     <xf numFmtId="0" fontId="16" fillId="28" borderId="0"/>
     <xf numFmtId="0" fontId="16" fillId="32" borderId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="12" borderId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="16" borderId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="20" borderId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="24" borderId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="28" borderId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="32" borderId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="12" borderId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="16" borderId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="20" borderId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="24" borderId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="28" borderId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="32" borderId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="12" borderId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="16" borderId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="20" borderId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="24" borderId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="28" borderId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="32" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
-  <cellStyles count="56">
+  <cellStyles count="77">
     <cellStyle name="20 % - Accent1 2" xfId="26" xr:uid="{00000000-0005-0000-0000-00001A000000}"/>
     <cellStyle name="20 % - Accent2 2" xfId="30" xr:uid="{00000000-0005-0000-0000-00001E000000}"/>
     <cellStyle name="20 % - Accent3 2" xfId="34" xr:uid="{00000000-0005-0000-0000-000022000000}"/>
@@ -566,22 +587,40 @@
     <cellStyle name="40 % - Accent6 2" xfId="47" xr:uid="{00000000-0005-0000-0000-00002F000000}"/>
     <cellStyle name="60 % - Accent1 2" xfId="2" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
     <cellStyle name="60 % - Accent1 3" xfId="28" xr:uid="{00000000-0005-0000-0000-00001C000000}"/>
-    <cellStyle name="60 % - Accent1 4" xfId="50" xr:uid="{00000000-0005-0000-0000-000054000000}"/>
+    <cellStyle name="60 % - Accent1 4" xfId="50" xr:uid="{00000000-0005-0000-0000-000032000000}"/>
+    <cellStyle name="60 % - Accent1 5" xfId="57" xr:uid="{00000000-0005-0000-0000-000039000000}"/>
+    <cellStyle name="60 % - Accent1 6" xfId="64" xr:uid="{00000000-0005-0000-0000-000040000000}"/>
+    <cellStyle name="60 % - Accent1 7" xfId="71" xr:uid="{00000000-0005-0000-0000-000069000000}"/>
     <cellStyle name="60 % - Accent2 2" xfId="3" xr:uid="{00000000-0005-0000-0000-000003000000}"/>
     <cellStyle name="60 % - Accent2 3" xfId="32" xr:uid="{00000000-0005-0000-0000-000020000000}"/>
-    <cellStyle name="60 % - Accent2 4" xfId="51" xr:uid="{00000000-0005-0000-0000-000055000000}"/>
+    <cellStyle name="60 % - Accent2 4" xfId="51" xr:uid="{00000000-0005-0000-0000-000033000000}"/>
+    <cellStyle name="60 % - Accent2 5" xfId="58" xr:uid="{00000000-0005-0000-0000-00003A000000}"/>
+    <cellStyle name="60 % - Accent2 6" xfId="65" xr:uid="{00000000-0005-0000-0000-000041000000}"/>
+    <cellStyle name="60 % - Accent2 7" xfId="72" xr:uid="{00000000-0005-0000-0000-00006A000000}"/>
     <cellStyle name="60 % - Accent3 2" xfId="4" xr:uid="{00000000-0005-0000-0000-000004000000}"/>
     <cellStyle name="60 % - Accent3 3" xfId="36" xr:uid="{00000000-0005-0000-0000-000024000000}"/>
-    <cellStyle name="60 % - Accent3 4" xfId="52" xr:uid="{00000000-0005-0000-0000-000056000000}"/>
+    <cellStyle name="60 % - Accent3 4" xfId="52" xr:uid="{00000000-0005-0000-0000-000034000000}"/>
+    <cellStyle name="60 % - Accent3 5" xfId="59" xr:uid="{00000000-0005-0000-0000-00003B000000}"/>
+    <cellStyle name="60 % - Accent3 6" xfId="66" xr:uid="{00000000-0005-0000-0000-000042000000}"/>
+    <cellStyle name="60 % - Accent3 7" xfId="73" xr:uid="{00000000-0005-0000-0000-00006B000000}"/>
     <cellStyle name="60 % - Accent4 2" xfId="5" xr:uid="{00000000-0005-0000-0000-000005000000}"/>
     <cellStyle name="60 % - Accent4 3" xfId="40" xr:uid="{00000000-0005-0000-0000-000028000000}"/>
-    <cellStyle name="60 % - Accent4 4" xfId="53" xr:uid="{00000000-0005-0000-0000-000057000000}"/>
+    <cellStyle name="60 % - Accent4 4" xfId="53" xr:uid="{00000000-0005-0000-0000-000035000000}"/>
+    <cellStyle name="60 % - Accent4 5" xfId="60" xr:uid="{00000000-0005-0000-0000-00003C000000}"/>
+    <cellStyle name="60 % - Accent4 6" xfId="67" xr:uid="{00000000-0005-0000-0000-000043000000}"/>
+    <cellStyle name="60 % - Accent4 7" xfId="74" xr:uid="{00000000-0005-0000-0000-00006C000000}"/>
     <cellStyle name="60 % - Accent5 2" xfId="6" xr:uid="{00000000-0005-0000-0000-000006000000}"/>
     <cellStyle name="60 % - Accent5 3" xfId="44" xr:uid="{00000000-0005-0000-0000-00002C000000}"/>
-    <cellStyle name="60 % - Accent5 4" xfId="54" xr:uid="{00000000-0005-0000-0000-000058000000}"/>
+    <cellStyle name="60 % - Accent5 4" xfId="54" xr:uid="{00000000-0005-0000-0000-000036000000}"/>
+    <cellStyle name="60 % - Accent5 5" xfId="61" xr:uid="{00000000-0005-0000-0000-00003D000000}"/>
+    <cellStyle name="60 % - Accent5 6" xfId="68" xr:uid="{00000000-0005-0000-0000-000044000000}"/>
+    <cellStyle name="60 % - Accent5 7" xfId="75" xr:uid="{00000000-0005-0000-0000-00006D000000}"/>
     <cellStyle name="60 % - Accent6 2" xfId="7" xr:uid="{00000000-0005-0000-0000-000007000000}"/>
     <cellStyle name="60 % - Accent6 3" xfId="48" xr:uid="{00000000-0005-0000-0000-000030000000}"/>
-    <cellStyle name="60 % - Accent6 4" xfId="55" xr:uid="{00000000-0005-0000-0000-000059000000}"/>
+    <cellStyle name="60 % - Accent6 4" xfId="55" xr:uid="{00000000-0005-0000-0000-000037000000}"/>
+    <cellStyle name="60 % - Accent6 5" xfId="62" xr:uid="{00000000-0005-0000-0000-00003E000000}"/>
+    <cellStyle name="60 % - Accent6 6" xfId="69" xr:uid="{00000000-0005-0000-0000-000045000000}"/>
+    <cellStyle name="60 % - Accent6 7" xfId="76" xr:uid="{00000000-0005-0000-0000-00006E000000}"/>
     <cellStyle name="Accent1 2" xfId="25" xr:uid="{00000000-0005-0000-0000-000019000000}"/>
     <cellStyle name="Accent2 2" xfId="29" xr:uid="{00000000-0005-0000-0000-00001D000000}"/>
     <cellStyle name="Accent3 2" xfId="33" xr:uid="{00000000-0005-0000-0000-000021000000}"/>
@@ -595,7 +634,10 @@
     <cellStyle name="Insatisfaisant 2" xfId="14" xr:uid="{00000000-0005-0000-0000-00000E000000}"/>
     <cellStyle name="Neutre 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
     <cellStyle name="Neutre 3" xfId="15" xr:uid="{00000000-0005-0000-0000-00000F000000}"/>
-    <cellStyle name="Neutre 4" xfId="49" xr:uid="{00000000-0005-0000-0000-000053000000}"/>
+    <cellStyle name="Neutre 4" xfId="49" xr:uid="{00000000-0005-0000-0000-000031000000}"/>
+    <cellStyle name="Neutre 5" xfId="56" xr:uid="{00000000-0005-0000-0000-000038000000}"/>
+    <cellStyle name="Neutre 6" xfId="63" xr:uid="{00000000-0005-0000-0000-00003F000000}"/>
+    <cellStyle name="Neutre 7" xfId="70" xr:uid="{00000000-0005-0000-0000-000068000000}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Note 2" xfId="22" xr:uid="{00000000-0005-0000-0000-000016000000}"/>
     <cellStyle name="Satisfaisant 2" xfId="13" xr:uid="{00000000-0005-0000-0000-00000D000000}"/>
@@ -926,6 +968,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="E1" s="1"/>
       <c r="F1" s="1"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">

</xml_diff>